<commit_message>
Removes Solar for All from 2025 to get closer to SEIA historical
</commit_message>
<xml_diff>
--- a/InputData/bldgs/BDESC/BAU Distribued Electricity Source Capacities.xlsx
+++ b/InputData/bldgs/BDESC/BAU Distribued Electricity Source Capacities.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OliviaAshmoore\Documents\Github Repos\eps-us\InputData\bldgs\BDESC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\bldgs\BDESC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E6E8EC5-5554-4F4F-A346-436352FFA6BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDD02FB4-E0CF-4FA4-A608-2ACFECDF4BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21030" yWindow="750" windowWidth="21600" windowHeight="12585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -12847,8 +12847,9 @@
       <c r="B1">
         <v>2024</v>
       </c>
-      <c r="C1">
-        <v>2025</v>
+      <c r="C1" s="57">
+        <f>C8-B8+'BDESC-rural-residential'!C8-'BDESC-rural-residential'!B8+'BDESC-commercial'!C8-'BDESC-commercial'!B8</f>
+        <v>7213.474999999984</v>
       </c>
       <c r="D1">
         <v>2026</v>
@@ -13504,9 +13505,9 @@
         <f>Calculations!D48+'Inflation Reduction Act'!C59</f>
         <v>33586.644085485314</v>
       </c>
-      <c r="C8" s="56">
-        <f>Calculations!E48+'Inflation Reduction Act'!D59</f>
-        <v>37908.465848613647</v>
+      <c r="C8" s="57">
+        <f>Calculations!E48</f>
+        <v>36072.861350926898</v>
       </c>
       <c r="D8" s="57">
         <f>Calculations!F48</f>
@@ -15833,9 +15834,9 @@
         <f>Calculations!D67+'Inflation Reduction Act'!C60</f>
         <v>7721.182914514693</v>
       </c>
-      <c r="C8" s="53">
-        <f>Calculations!E67+'Inflation Reduction Act'!D60</f>
-        <v>8714.7199964604661</v>
+      <c r="C8">
+        <f>Calculations!E67</f>
+        <v>8292.7356490730999</v>
       </c>
       <c r="D8">
         <f>Calculations!F67</f>

</xml_diff>

<commit_message>
Adds existing BTM gas to BDESC; adds planned gas to BPMCCS; lowers wind CSC to 0.1 through 2030
</commit_message>
<xml_diff>
--- a/InputData/bldgs/BDESC/BAU Distribued Electricity Source Capacities.xlsx
+++ b/InputData/bldgs/BDESC/BAU Distribued Electricity Source Capacities.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\bldgs\BDESC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{804AE395-CB52-412A-8281-449A450ABD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E568A12B-05DA-4807-A2BF-B044209A26FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2046" uniqueCount="996">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2050" uniqueCount="999">
   <si>
     <t>BDESC BAU Distributed Electricity Source Capacity</t>
   </si>
@@ -3038,55 +3038,75 @@
     <t>Behind-the-meter Data Center Gas Plants</t>
   </si>
   <si>
-    <t>Cleanview</t>
-  </si>
-  <si>
-    <t>Bypassing the Grid: How Data Center Developers Are Building Their Own Power Plants</t>
-  </si>
-  <si>
-    <t>https://cleanview.co/reports/behind-the-meter-data-centers</t>
-  </si>
-  <si>
-    <t>Cleanview's 2026 data finds 90 GW of announced capacity planned for behind-the-meter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gas capacity, with 82 GW of that announced since Q1 2025. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">"Of the roughly 90 GW of generation capacity we've identified across all projects, only </t>
-  </si>
-  <si>
-    <t xml:space="preserve">about 2 GW is actually operating today—2.5% of the total. 1.2% is under construction. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Another 36% has been permitted, and the remaining 60% exists only as announcements </t>
-  </si>
-  <si>
-    <t>or early-stage plans.</t>
-  </si>
-  <si>
-    <t>GW total</t>
-  </si>
-  <si>
-    <t>permitted</t>
-  </si>
-  <si>
-    <t>online</t>
-  </si>
-  <si>
-    <t>under construction</t>
-  </si>
-  <si>
-    <t>announced</t>
-  </si>
-  <si>
-    <t>We add the under-construction and permitted capacity to AEO forecasts, assuming that</t>
-  </si>
-  <si>
-    <t>all will come online by 2030 to meet the first wave of AI data center buildout in the U.S.</t>
-  </si>
-  <si>
-    <t>new capacity</t>
+    <r>
+      <t>Table 3.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13.5"/>
+        <color rgb="FF161400"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> Overall Behind-the-Meter Effective Capacity Growth by Region Out to 2030 (GW)</t>
+    </r>
+  </si>
+  <si>
+    <t>Actual</t>
+  </si>
+  <si>
+    <t>Forecast</t>
+  </si>
+  <si>
+    <t>ISO regions</t>
+  </si>
+  <si>
+    <t>CAISO</t>
+  </si>
+  <si>
+    <t>ERCOT</t>
+  </si>
+  <si>
+    <t>NE-ISO</t>
+  </si>
+  <si>
+    <t>MISO</t>
+  </si>
+  <si>
+    <t>NY-ISO</t>
+  </si>
+  <si>
+    <t>PJM</t>
+  </si>
+  <si>
+    <t>SPP</t>
+  </si>
+  <si>
+    <t>Non-ISO regions</t>
+  </si>
+  <si>
+    <t>Annual incremental</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>RAND has estimated the behind the meter capacity to support data centers through 2030.</t>
+  </si>
+  <si>
+    <t>We assume 100% of this gas.</t>
+  </si>
+  <si>
+    <t>We add this forecasted capacity to AEO forecasts, which isn't capturing this trend</t>
+  </si>
+  <si>
+    <t>RAND</t>
+  </si>
+  <si>
+    <t>https://www.rand.org/pubs/research_briefs/RBA3845-1.html</t>
+  </si>
+  <si>
+    <t>How Much More Power Can the U.S. Grid Provide for AI?</t>
   </si>
 </sst>
 </file>
@@ -3102,7 +3122,7 @@
     <numFmt numFmtId="168" formatCode="0.00000000000"/>
     <numFmt numFmtId="169" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="30" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3287,6 +3307,32 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="13.5"/>
+      <color rgb="FF161400"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13.5"/>
+      <color rgb="FF2D2B19"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF2D2B19"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF2D2B19"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="20">
     <fill>
@@ -3403,7 +3449,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -3580,6 +3626,94 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color rgb="FF2D2B19"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFD0D0CC"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color rgb="FF2D2B19"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFD0D0CC"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFD0D0CC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFD0D0CC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFD0D0CC"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color rgb="FF2D2B19"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thick">
+        <color rgb="FF2D2B19"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFD0D0CC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFD0D0CC"/>
+      </right>
+      <top style="thick">
+        <color rgb="FF2D2B19"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFD0D0CC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFD0D0CC"/>
+      </left>
+      <right/>
+      <top style="thick">
+        <color rgb="FF2D2B19"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFD0D0CC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -3615,7 +3749,7 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3744,11 +3878,27 @@
     <xf numFmtId="0" fontId="24" fillId="18" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -3756,7 +3906,13 @@
     <xf numFmtId="0" fontId="25" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="18" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3779,10 +3935,33 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="20">
     <cellStyle name="60% - Accent1 2" xfId="12" xr:uid="{00000000-0005-0000-0000-00002E000000}"/>
@@ -11710,7 +11889,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>979</v>
+        <v>996</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -11720,12 +11899,12 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
-        <v>980</v>
+        <v>998</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B24" s="18" t="s">
-        <v>981</v>
+        <v>997</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -23435,689 +23614,774 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{858104B2-5734-4794-B2D1-CAE7717AD060}">
-  <dimension ref="B2:AB26"/>
+  <dimension ref="B2:AC27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B2" s="79" t="s">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>993</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>994</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="B7" s="65" t="s">
+        <v>979</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="87"/>
+      <c r="C9" s="89" t="s">
+        <v>980</v>
+      </c>
+      <c r="D9" s="89"/>
+      <c r="E9" s="90"/>
+      <c r="F9" s="91" t="s">
+        <v>981</v>
+      </c>
+      <c r="G9" s="89"/>
+      <c r="H9" s="89"/>
+      <c r="I9" s="89"/>
+    </row>
+    <row r="10" spans="2:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="88"/>
+      <c r="C10" s="66">
+        <v>2024</v>
+      </c>
+      <c r="D10" s="66">
+        <v>2025</v>
+      </c>
+      <c r="E10" s="67">
+        <v>2026</v>
+      </c>
+      <c r="F10" s="66">
+        <v>2027</v>
+      </c>
+      <c r="G10" s="66">
+        <v>2028</v>
+      </c>
+      <c r="H10" s="66">
+        <v>2029</v>
+      </c>
+      <c r="I10" s="66">
+        <v>2030</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="92" t="s">
         <v>982</v>
       </c>
-    </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
+      <c r="C11" s="92"/>
+      <c r="D11" s="92"/>
+      <c r="E11" s="93"/>
+      <c r="F11" s="94"/>
+      <c r="G11" s="95"/>
+      <c r="H11" s="95"/>
+      <c r="I11" s="95"/>
+    </row>
+    <row r="12" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="68" t="s">
         <v>983</v>
       </c>
-    </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
+      <c r="C12" s="69">
+        <v>3</v>
+      </c>
+      <c r="D12" s="69">
+        <v>3.1</v>
+      </c>
+      <c r="E12" s="70">
+        <v>3.2</v>
+      </c>
+      <c r="F12" s="69">
+        <v>3.3</v>
+      </c>
+      <c r="G12" s="69">
+        <v>3.4</v>
+      </c>
+      <c r="H12" s="69">
+        <v>3.5</v>
+      </c>
+      <c r="I12" s="69">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="68" t="s">
         <v>984</v>
       </c>
-    </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B6" t="s">
+      <c r="C13" s="69">
+        <v>2</v>
+      </c>
+      <c r="D13" s="69">
+        <v>3.3</v>
+      </c>
+      <c r="E13" s="70">
+        <v>4.7</v>
+      </c>
+      <c r="F13" s="69">
+        <v>4.8</v>
+      </c>
+      <c r="G13" s="69">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="H13" s="69">
+        <v>6.9</v>
+      </c>
+      <c r="I13" s="69">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="68" t="s">
         <v>985</v>
       </c>
-    </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B7" t="s">
+      <c r="C14" s="69">
+        <v>0.2</v>
+      </c>
+      <c r="D14" s="69">
+        <v>0.2</v>
+      </c>
+      <c r="E14" s="70">
+        <v>0.2</v>
+      </c>
+      <c r="F14" s="69">
+        <v>0.4</v>
+      </c>
+      <c r="G14" s="69">
+        <v>0.6</v>
+      </c>
+      <c r="H14" s="69">
+        <v>0.8</v>
+      </c>
+      <c r="I14" s="69">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="68" t="s">
         <v>986</v>
       </c>
-    </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
+      <c r="C15" s="69">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="D15" s="69">
+        <v>2.5</v>
+      </c>
+      <c r="E15" s="70">
+        <v>2.9</v>
+      </c>
+      <c r="F15" s="69">
+        <v>3.9</v>
+      </c>
+      <c r="G15" s="69">
+        <v>5</v>
+      </c>
+      <c r="H15" s="69">
+        <v>8.1</v>
+      </c>
+      <c r="I15" s="69">
+        <v>11.2</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="68" t="s">
         <v>987</v>
       </c>
-    </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B10">
-        <v>90</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="C16" s="69">
+        <v>0.8</v>
+      </c>
+      <c r="D16" s="69">
+        <v>1.6</v>
+      </c>
+      <c r="E16" s="70">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="F16" s="69">
+        <v>2.6</v>
+      </c>
+      <c r="G16" s="69">
+        <v>2.8</v>
+      </c>
+      <c r="H16" s="69">
+        <v>3</v>
+      </c>
+      <c r="I16" s="69">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="17" spans="2:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="68" t="s">
         <v>988</v>
       </c>
-    </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B11" s="81">
-        <v>2.5000000000000001E-2</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="C17" s="69">
+        <v>0.9</v>
+      </c>
+      <c r="D17" s="69">
+        <v>1.8</v>
+      </c>
+      <c r="E17" s="70">
+        <v>2.6</v>
+      </c>
+      <c r="F17" s="69">
+        <v>2.9</v>
+      </c>
+      <c r="G17" s="69">
+        <v>3.2</v>
+      </c>
+      <c r="H17" s="69">
+        <v>3.9</v>
+      </c>
+      <c r="I17" s="69">
+        <v>4.7</v>
+      </c>
+    </row>
+    <row r="18" spans="2:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="68" t="s">
+        <v>989</v>
+      </c>
+      <c r="C18" s="69">
+        <v>0.5</v>
+      </c>
+      <c r="D18" s="69">
+        <v>0.6</v>
+      </c>
+      <c r="E18" s="70">
+        <v>0.7</v>
+      </c>
+      <c r="F18" s="69">
+        <v>0.9</v>
+      </c>
+      <c r="G18" s="69">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="H18" s="69">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="I18" s="69">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="19" spans="2:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="68" t="s">
         <v>990</v>
       </c>
-    </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B12" s="16">
-        <v>1.2E-2</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="C19" s="69">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="D19" s="69">
+        <v>3.5</v>
+      </c>
+      <c r="E19" s="70">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="F19" s="69">
+        <v>6</v>
+      </c>
+      <c r="G19" s="69">
+        <v>7.3</v>
+      </c>
+      <c r="H19" s="69">
+        <v>9.6999999999999993</v>
+      </c>
+      <c r="I19" s="69">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="2:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="68" t="s">
         <v>991</v>
       </c>
-    </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B13" s="80">
-        <v>0.36</v>
-      </c>
-      <c r="C13" t="s">
-        <v>989</v>
-      </c>
-    </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B14" s="80">
-        <v>0.6</v>
-      </c>
-      <c r="C14" t="s">
+      <c r="C20" s="69" t="s">
         <v>992</v>
       </c>
-    </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B16" t="s">
-        <v>993</v>
-      </c>
-    </row>
-    <row r="17" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B17" t="s">
-        <v>994</v>
-      </c>
-    </row>
-    <row r="19" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="C19">
+      <c r="D20" s="69">
+        <v>4.7</v>
+      </c>
+      <c r="E20" s="70">
+        <v>4.7</v>
+      </c>
+      <c r="F20" s="69">
+        <v>3.5</v>
+      </c>
+      <c r="G20" s="69">
+        <v>3.5</v>
+      </c>
+      <c r="H20" s="69">
+        <v>10</v>
+      </c>
+      <c r="I20" s="69">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="2:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="71" t="s">
+        <v>37</v>
+      </c>
+      <c r="C21" s="69">
+        <v>12</v>
+      </c>
+      <c r="D21" s="69">
+        <v>17</v>
+      </c>
+      <c r="E21" s="70">
+        <v>21</v>
+      </c>
+      <c r="F21" s="69">
+        <v>25</v>
+      </c>
+      <c r="G21" s="69">
+        <v>29</v>
+      </c>
+      <c r="H21" s="69">
+        <v>39</v>
+      </c>
+      <c r="I21" s="69">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="24" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="C24">
+        <v>2024</v>
+      </c>
+      <c r="D24">
         <v>2025</v>
       </c>
-      <c r="D19">
+      <c r="E24">
         <v>2026</v>
       </c>
-      <c r="E19">
+      <c r="F24">
         <v>2027</v>
       </c>
-      <c r="F19">
+      <c r="G24">
         <v>2028</v>
       </c>
-      <c r="G19">
+      <c r="H24">
         <v>2029</v>
       </c>
-      <c r="H19">
+      <c r="I24">
         <v>2030</v>
       </c>
-      <c r="I19">
+      <c r="J24">
         <v>2031</v>
       </c>
-      <c r="J19">
+      <c r="K24">
         <v>2032</v>
       </c>
-      <c r="K19">
+      <c r="L24">
         <v>2033</v>
       </c>
-      <c r="L19">
+      <c r="M24">
         <v>2034</v>
       </c>
-      <c r="M19">
+      <c r="N24">
         <v>2035</v>
       </c>
-      <c r="N19">
+      <c r="O24">
         <v>2036</v>
       </c>
-      <c r="O19">
+      <c r="P24">
         <v>2037</v>
       </c>
-      <c r="P19">
+      <c r="Q24">
         <v>2038</v>
       </c>
-      <c r="Q19">
+      <c r="R24">
         <v>2039</v>
       </c>
-      <c r="R19">
+      <c r="S24">
         <v>2040</v>
       </c>
-      <c r="S19">
+      <c r="T24">
         <v>2041</v>
       </c>
-      <c r="T19">
+      <c r="U24">
         <v>2042</v>
       </c>
-      <c r="U19">
+      <c r="V24">
         <v>2043</v>
       </c>
-      <c r="V19">
+      <c r="W24">
         <v>2044</v>
       </c>
-      <c r="W19">
+      <c r="X24">
         <v>2045</v>
       </c>
-      <c r="X19">
+      <c r="Y24">
         <v>2046</v>
       </c>
-      <c r="Y19">
+      <c r="Z24">
         <v>2047</v>
       </c>
-      <c r="Z19">
+      <c r="AA24">
         <v>2048</v>
       </c>
-      <c r="AA19">
+      <c r="AB24">
         <v>2049</v>
       </c>
-      <c r="AB19">
+      <c r="AC24">
         <v>2050</v>
       </c>
     </row>
-    <row r="20" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B20" t="s">
-        <v>995</v>
-      </c>
-      <c r="C20">
-        <v>0</v>
-      </c>
-      <c r="D20">
-        <f>$B$10*$B$13/5+C20</f>
-        <v>6.4799999999999995</v>
-      </c>
-      <c r="E20">
-        <f>$B$10*$B$13/5+D20</f>
-        <v>12.959999999999999</v>
-      </c>
-      <c r="F20">
-        <f t="shared" ref="F20:H20" si="0">$B$10*$B$13/5+E20</f>
-        <v>19.439999999999998</v>
-      </c>
-      <c r="G20">
-        <f t="shared" si="0"/>
-        <v>25.919999999999998</v>
-      </c>
-      <c r="H20">
-        <f t="shared" si="0"/>
-        <v>32.4</v>
-      </c>
-      <c r="I20">
-        <f>H20</f>
-        <v>32.4</v>
-      </c>
-      <c r="J20">
-        <f t="shared" ref="J20:AB20" si="1">I20</f>
-        <v>32.4</v>
-      </c>
-      <c r="K20">
-        <f t="shared" si="1"/>
-        <v>32.4</v>
-      </c>
-      <c r="L20">
-        <f t="shared" si="1"/>
-        <v>32.4</v>
-      </c>
-      <c r="M20">
-        <f t="shared" si="1"/>
-        <v>32.4</v>
-      </c>
-      <c r="N20">
-        <f t="shared" si="1"/>
-        <v>32.4</v>
-      </c>
-      <c r="O20">
-        <f t="shared" si="1"/>
-        <v>32.4</v>
-      </c>
-      <c r="P20">
-        <f t="shared" si="1"/>
-        <v>32.4</v>
-      </c>
-      <c r="Q20">
-        <f t="shared" si="1"/>
-        <v>32.4</v>
-      </c>
-      <c r="R20">
-        <f t="shared" si="1"/>
-        <v>32.4</v>
-      </c>
-      <c r="S20">
-        <f t="shared" si="1"/>
-        <v>32.4</v>
-      </c>
-      <c r="T20">
-        <f t="shared" si="1"/>
-        <v>32.4</v>
-      </c>
-      <c r="U20">
-        <f t="shared" si="1"/>
-        <v>32.4</v>
-      </c>
-      <c r="V20">
-        <f t="shared" si="1"/>
-        <v>32.4</v>
-      </c>
-      <c r="W20">
-        <f t="shared" si="1"/>
-        <v>32.4</v>
-      </c>
-      <c r="X20">
-        <f t="shared" si="1"/>
-        <v>32.4</v>
-      </c>
-      <c r="Y20">
-        <f t="shared" si="1"/>
-        <v>32.4</v>
-      </c>
-      <c r="Z20">
-        <f t="shared" si="1"/>
-        <v>32.4</v>
-      </c>
-      <c r="AA20">
-        <f t="shared" si="1"/>
-        <v>32.4</v>
-      </c>
-      <c r="AB20">
-        <f t="shared" si="1"/>
-        <v>32.4</v>
-      </c>
-    </row>
-    <row r="23" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="C23">
-        <v>2025</v>
-      </c>
-      <c r="D23">
-        <v>2026</v>
-      </c>
-      <c r="E23">
-        <v>2027</v>
-      </c>
-      <c r="F23">
-        <v>2028</v>
-      </c>
-      <c r="G23">
-        <v>2029</v>
-      </c>
-      <c r="H23">
-        <v>2030</v>
-      </c>
-      <c r="I23">
-        <v>2031</v>
-      </c>
-      <c r="J23">
-        <v>2032</v>
-      </c>
-      <c r="K23">
-        <v>2033</v>
-      </c>
-      <c r="L23">
-        <v>2034</v>
-      </c>
-      <c r="M23">
-        <v>2035</v>
-      </c>
-      <c r="N23">
-        <v>2036</v>
-      </c>
-      <c r="O23">
-        <v>2037</v>
-      </c>
-      <c r="P23">
-        <v>2038</v>
-      </c>
-      <c r="Q23">
-        <v>2039</v>
-      </c>
-      <c r="R23">
-        <v>2040</v>
-      </c>
-      <c r="S23">
-        <v>2041</v>
-      </c>
-      <c r="T23">
-        <v>2042</v>
-      </c>
-      <c r="U23">
-        <v>2043</v>
-      </c>
-      <c r="V23">
-        <v>2044</v>
-      </c>
-      <c r="W23">
-        <v>2045</v>
-      </c>
-      <c r="X23">
-        <v>2046</v>
-      </c>
-      <c r="Y23">
-        <v>2047</v>
-      </c>
-      <c r="Z23">
-        <v>2048</v>
-      </c>
-      <c r="AA23">
-        <v>2049</v>
-      </c>
-      <c r="AB23">
-        <v>2050</v>
-      </c>
-    </row>
-    <row r="24" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B24" s="1" t="s">
+    <row r="25" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="B25" s="1" t="s">
         <v>548</v>
       </c>
-      <c r="C24">
+      <c r="C25">
+        <f>Calculations!D44</f>
+        <v>1.4025661782562939</v>
+      </c>
+      <c r="D25">
         <f>Calculations!E44</f>
         <v>0.41060633044604544</v>
       </c>
-      <c r="D24">
+      <c r="E25">
         <f>Calculations!F44</f>
         <v>0.89845543592649557</v>
       </c>
-      <c r="E24">
+      <c r="F25">
         <f>Calculations!G44</f>
         <v>1.3732952319274669</v>
       </c>
-      <c r="F24">
+      <c r="G25">
         <f>Calculations!H44</f>
         <v>1.3838652958795432</v>
       </c>
-      <c r="G24">
+      <c r="H25">
         <f>Calculations!I44</f>
         <v>1.3944353598316197</v>
       </c>
-      <c r="H24">
+      <c r="I25">
         <f>Calculations!J44</f>
         <v>2.0562839796000971</v>
       </c>
-      <c r="I24">
+      <c r="J25">
         <f>Calculations!K44</f>
         <v>2.9401039423621791</v>
       </c>
-      <c r="J24">
+      <c r="K25">
         <f>Calculations!L44</f>
         <v>3.8515686877681534</v>
       </c>
-      <c r="K24">
+      <c r="L25">
         <f>Calculations!M44</f>
         <v>4.5605760543997409</v>
       </c>
-      <c r="L24">
+      <c r="M25">
         <f>Calculations!N44</f>
         <v>5.449274508216627</v>
       </c>
-      <c r="M24">
+      <c r="N25">
         <f>Calculations!O44</f>
         <v>5.459844572168703</v>
       </c>
-      <c r="N24">
+      <c r="O25">
         <f>Calculations!P44</f>
         <v>5.4704146361207799</v>
       </c>
-      <c r="O24">
+      <c r="P25">
         <f>Calculations!Q44</f>
         <v>5.480984700072856</v>
       </c>
-      <c r="P24">
+      <c r="Q25">
         <f>Calculations!R44</f>
         <v>5.4915547640249329</v>
       </c>
-      <c r="Q24">
+      <c r="R25">
         <f>Calculations!S44</f>
         <v>5.5029379098194759</v>
       </c>
-      <c r="R24">
+      <c r="S25">
         <f>Calculations!T44</f>
         <v>5.5143210556140208</v>
       </c>
-      <c r="S24">
+      <c r="T25">
         <f>Calculations!U44</f>
         <v>5.5273303650934995</v>
       </c>
-      <c r="T24">
+      <c r="U25">
         <f>Calculations!V44</f>
         <v>5.5444050837853149</v>
       </c>
-      <c r="U24">
+      <c r="V25">
         <f>Calculations!W44</f>
         <v>5.5679844572168697</v>
       </c>
-      <c r="V24">
+      <c r="W25">
         <f>Calculations!X44</f>
         <v>5.6053862219703712</v>
       </c>
-      <c r="W24">
+      <c r="X25">
         <f>Calculations!Y44</f>
         <v>5.6696196875252971</v>
       </c>
-      <c r="X24">
+      <c r="Y25">
         <f>Calculations!Z44</f>
         <v>5.7818249817858005</v>
       </c>
-      <c r="Y24">
+      <c r="Z25">
         <f>Calculations!AA44</f>
         <v>5.8940302760463048</v>
       </c>
-      <c r="Z24">
+      <c r="AA25">
         <f>Calculations!AB44</f>
         <v>6.0070486521492752</v>
       </c>
-      <c r="AA24">
+      <c r="AB25">
         <f>Calculations!AC44</f>
         <v>6.1208801100947134</v>
       </c>
-      <c r="AB24">
+      <c r="AC25">
         <f>Calculations!AD44</f>
         <v>6.2355246498826196</v>
       </c>
     </row>
-    <row r="25" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B25" s="1" t="s">
+    <row r="26" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="B26" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="C25">
+      <c r="C26">
+        <f>Calculations!D63</f>
+        <v>0.32243382174370594</v>
+      </c>
+      <c r="D26">
         <f>Calculations!E63</f>
         <v>9.4393669553954507E-2</v>
       </c>
-      <c r="D25">
+      <c r="E26">
         <f>Calculations!F63</f>
         <v>0.20654456407350441</v>
       </c>
-      <c r="E25">
+      <c r="F26">
         <f>Calculations!G63</f>
         <v>0.31570476807253295</v>
       </c>
-      <c r="F25">
+      <c r="G26">
         <f>Calculations!H63</f>
         <v>0.31813470412045658</v>
       </c>
-      <c r="G25">
+      <c r="H26">
         <f>Calculations!I63</f>
         <v>0.32056464016838015</v>
       </c>
-      <c r="H25">
+      <c r="I26">
         <f>Calculations!J63</f>
         <v>0.47271602039990285</v>
       </c>
-      <c r="I25">
+      <c r="J26">
         <f>Calculations!K63</f>
         <v>0.67589605763782079</v>
       </c>
-      <c r="J25">
+      <c r="K26">
         <f>Calculations!L63</f>
         <v>0.88543131223184646</v>
       </c>
-      <c r="K25">
+      <c r="L26">
         <f>Calculations!M63</f>
         <v>1.0484239456002591</v>
       </c>
-      <c r="L25">
+      <c r="M26">
         <f>Calculations!N63</f>
         <v>1.2527254917833723</v>
       </c>
-      <c r="M25">
+      <c r="N26">
         <f>Calculations!O63</f>
         <v>1.255155427831296</v>
       </c>
-      <c r="N25">
+      <c r="O26">
         <f>Calculations!P63</f>
         <v>1.2575853638792196</v>
       </c>
-      <c r="O25">
+      <c r="P26">
         <f>Calculations!Q63</f>
         <v>1.2600152999271432</v>
       </c>
-      <c r="P25">
+      <c r="Q26">
         <f>Calculations!R63</f>
         <v>1.2624452359750666</v>
       </c>
-      <c r="Q25">
+      <c r="R26">
         <f>Calculations!S63</f>
         <v>1.265062090180523</v>
       </c>
-      <c r="R25">
+      <c r="S26">
         <f>Calculations!T63</f>
         <v>1.2676789443859791</v>
       </c>
-      <c r="S25">
+      <c r="T26">
         <f>Calculations!U63</f>
         <v>1.2706696349065005</v>
       </c>
-      <c r="T25">
+      <c r="U26">
         <f>Calculations!V63</f>
         <v>1.2745949162146848</v>
       </c>
-      <c r="U25">
+      <c r="V26">
         <f>Calculations!W63</f>
         <v>1.2800155427831297</v>
       </c>
-      <c r="V25">
+      <c r="W26">
         <f>Calculations!X63</f>
         <v>1.2886137780296285</v>
       </c>
-      <c r="W25">
+      <c r="X26">
         <f>Calculations!Y63</f>
         <v>1.3033803124747023</v>
       </c>
-      <c r="X25">
+      <c r="Y26">
         <f>Calculations!Z63</f>
         <v>1.329175018214199</v>
       </c>
-      <c r="Y25">
+      <c r="Z26">
         <f>Calculations!AA63</f>
         <v>1.3549697239536955</v>
       </c>
-      <c r="Z25">
+      <c r="AA26">
         <f>Calculations!AB63</f>
         <v>1.3809513478507245</v>
       </c>
-      <c r="AA25">
+      <c r="AB26">
         <f>Calculations!AC63</f>
         <v>1.4071198899052861</v>
       </c>
-      <c r="AB25">
+      <c r="AC26">
         <f>Calculations!AD63</f>
         <v>1.4334753501173803</v>
       </c>
     </row>
-    <row r="26" spans="2:28" x14ac:dyDescent="0.25">
-      <c r="B26" s="1" t="s">
+    <row r="27" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="B27" s="1" t="s">
         <v>555</v>
       </c>
-      <c r="C26">
-        <f>Calculations!E84</f>
-        <v>1508.008</v>
-      </c>
-      <c r="D26">
-        <f>Calculations!F84+D20*1000</f>
-        <v>8020.9689999999991</v>
-      </c>
-      <c r="E26">
-        <f>Calculations!G84+E20*1000</f>
-        <v>14519.124999999998</v>
-      </c>
-      <c r="F26">
-        <f>Calculations!H84+F20*1000</f>
-        <v>21016.868999999995</v>
-      </c>
-      <c r="G26">
-        <f>Calculations!I84+G20*1000</f>
-        <v>27515.394999999997</v>
-      </c>
-      <c r="H26">
-        <f>Calculations!J84+H20*1000</f>
-        <v>34015.290999999997</v>
-      </c>
-      <c r="I26">
-        <f>Calculations!K84+I20*1000</f>
-        <v>34034.760999999999</v>
-      </c>
-      <c r="J26">
-        <f>Calculations!L84+J20*1000</f>
-        <v>34055.343999999997</v>
-      </c>
-      <c r="K26">
-        <f>Calculations!M84+K20*1000</f>
-        <v>34076.552000000003</v>
-      </c>
-      <c r="L26">
-        <f>Calculations!N84+L20*1000</f>
-        <v>34100.095000000001</v>
-      </c>
-      <c r="M26">
-        <f>Calculations!O84+M20*1000</f>
-        <v>34122.014000000003</v>
-      </c>
-      <c r="N26">
-        <f>Calculations!P84+N20*1000</f>
-        <v>34144.811999999998</v>
-      </c>
-      <c r="O26">
-        <f>Calculations!Q84+O20*1000</f>
-        <v>34169.997000000003</v>
-      </c>
-      <c r="P26">
-        <f>Calculations!R84+P20*1000</f>
-        <v>34193.459000000003</v>
-      </c>
-      <c r="Q26">
-        <f>Calculations!S84+Q20*1000</f>
-        <v>34216.315999999999</v>
-      </c>
-      <c r="R26">
-        <f>Calculations!T84+R20*1000</f>
-        <v>34238.228000000003</v>
-      </c>
-      <c r="S26">
-        <f>Calculations!U84+S20*1000</f>
-        <v>34258.498999999996</v>
-      </c>
-      <c r="T26">
-        <f>Calculations!V84+T20*1000</f>
-        <v>34281.084999999999</v>
-      </c>
-      <c r="U26">
-        <f>Calculations!W84+U20*1000</f>
-        <v>34301.161999999997</v>
-      </c>
-      <c r="V26">
-        <f>Calculations!X84+V20*1000</f>
-        <v>34321.178</v>
-      </c>
-      <c r="W26">
-        <f>Calculations!Y84+W20*1000</f>
-        <v>34340.084000000003</v>
-      </c>
-      <c r="X26">
-        <f>Calculations!Z84+X20*1000</f>
-        <v>34359.432999999997</v>
-      </c>
-      <c r="Y26">
-        <f>Calculations!AA84+Y20*1000</f>
-        <v>34379.940999999999</v>
-      </c>
-      <c r="Z26">
-        <f>Calculations!AB84+Z20*1000</f>
-        <v>34400.097000000002</v>
-      </c>
-      <c r="AA26">
-        <f>Calculations!AC84+AA20*1000</f>
-        <v>34419.017999999996</v>
-      </c>
-      <c r="AB26">
-        <f>Calculations!AD84+AB20*1000</f>
-        <v>34439.06</v>
+      <c r="C27">
+        <f>Calculations!D84+C21*1000</f>
+        <v>13468.725</v>
+      </c>
+      <c r="D27">
+        <f>Calculations!E84+D21*1000</f>
+        <v>18508.008000000002</v>
+      </c>
+      <c r="E27">
+        <f>Calculations!F84+E21*1000</f>
+        <v>22540.969000000001</v>
+      </c>
+      <c r="F27">
+        <f>Calculations!G84+F21*1000</f>
+        <v>26559.125</v>
+      </c>
+      <c r="G27">
+        <f>Calculations!H84+G21*1000</f>
+        <v>30576.868999999999</v>
+      </c>
+      <c r="H27">
+        <f>Calculations!I84+H21*1000</f>
+        <v>40595.394999999997</v>
+      </c>
+      <c r="I27">
+        <f>Calculations!J84+I21*1000</f>
+        <v>50615.290999999997</v>
+      </c>
+      <c r="J27">
+        <f>Calculations!K84+$I$21*1000</f>
+        <v>50634.760999999999</v>
+      </c>
+      <c r="K27">
+        <f>Calculations!L84+$I$21*1000</f>
+        <v>50655.343999999997</v>
+      </c>
+      <c r="L27">
+        <f>Calculations!M84+$I$21*1000</f>
+        <v>50676.552000000003</v>
+      </c>
+      <c r="M27">
+        <f>Calculations!N84+$I$21*1000</f>
+        <v>50700.095000000001</v>
+      </c>
+      <c r="N27">
+        <f>Calculations!O84+$I$21*1000</f>
+        <v>50722.014000000003</v>
+      </c>
+      <c r="O27">
+        <f>Calculations!P84+$I$21*1000</f>
+        <v>50744.811999999998</v>
+      </c>
+      <c r="P27">
+        <f>Calculations!Q84+$I$21*1000</f>
+        <v>50769.997000000003</v>
+      </c>
+      <c r="Q27">
+        <f>Calculations!R84+$I$21*1000</f>
+        <v>50793.459000000003</v>
+      </c>
+      <c r="R27">
+        <f>Calculations!S84+$I$21*1000</f>
+        <v>50816.315999999999</v>
+      </c>
+      <c r="S27">
+        <f>Calculations!T84+$I$21*1000</f>
+        <v>50838.228000000003</v>
+      </c>
+      <c r="T27">
+        <f>Calculations!U84+$I$21*1000</f>
+        <v>50858.498999999996</v>
+      </c>
+      <c r="U27">
+        <f>Calculations!V84+$I$21*1000</f>
+        <v>50881.084999999999</v>
+      </c>
+      <c r="V27">
+        <f>Calculations!W84+$I$21*1000</f>
+        <v>50901.161999999997</v>
+      </c>
+      <c r="W27">
+        <f>Calculations!X84+$I$21*1000</f>
+        <v>50921.178</v>
+      </c>
+      <c r="X27">
+        <f>Calculations!Y84+$I$21*1000</f>
+        <v>50940.084000000003</v>
+      </c>
+      <c r="Y27">
+        <f>Calculations!Z84+$I$21*1000</f>
+        <v>50959.432999999997</v>
+      </c>
+      <c r="Z27">
+        <f>Calculations!AA84+$I$21*1000</f>
+        <v>50979.940999999999</v>
+      </c>
+      <c r="AA27">
+        <f>Calculations!AB84+$I$21*1000</f>
+        <v>51000.097000000002</v>
+      </c>
+      <c r="AB27">
+        <f>Calculations!AC84+$I$21*1000</f>
+        <v>51019.017999999996</v>
+      </c>
+      <c r="AC27">
+        <f>Calculations!AD84+$I$21*1000</f>
+        <v>51039.06</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="F9:I9"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="F11:I11"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -29287,109 +29551,109 @@
         <f>Calculations!D84</f>
         <v>1468.7250000000001</v>
       </c>
-      <c r="C4" s="82">
-        <f>'Data Center Gas'!C26</f>
-        <v>1508.008</v>
-      </c>
-      <c r="D4" s="82">
-        <f>'Data Center Gas'!D26</f>
-        <v>8020.9689999999991</v>
-      </c>
-      <c r="E4" s="82">
-        <f>'Data Center Gas'!E26</f>
-        <v>14519.124999999998</v>
-      </c>
-      <c r="F4" s="82">
-        <f>'Data Center Gas'!F26</f>
-        <v>21016.868999999995</v>
-      </c>
-      <c r="G4" s="82">
-        <f>'Data Center Gas'!G26</f>
-        <v>27515.394999999997</v>
-      </c>
-      <c r="H4" s="82">
-        <f>'Data Center Gas'!H26</f>
-        <v>34015.290999999997</v>
-      </c>
-      <c r="I4" s="82">
-        <f>'Data Center Gas'!I26</f>
-        <v>34034.760999999999</v>
-      </c>
-      <c r="J4" s="82">
-        <f>'Data Center Gas'!J26</f>
-        <v>34055.343999999997</v>
-      </c>
-      <c r="K4" s="82">
-        <f>'Data Center Gas'!K26</f>
-        <v>34076.552000000003</v>
-      </c>
-      <c r="L4" s="82">
-        <f>'Data Center Gas'!L26</f>
-        <v>34100.095000000001</v>
-      </c>
-      <c r="M4" s="82">
-        <f>'Data Center Gas'!M26</f>
-        <v>34122.014000000003</v>
-      </c>
-      <c r="N4" s="82">
-        <f>'Data Center Gas'!N26</f>
-        <v>34144.811999999998</v>
-      </c>
-      <c r="O4" s="82">
-        <f>'Data Center Gas'!O26</f>
-        <v>34169.997000000003</v>
-      </c>
-      <c r="P4" s="82">
-        <f>'Data Center Gas'!P26</f>
-        <v>34193.459000000003</v>
-      </c>
-      <c r="Q4" s="82">
-        <f>'Data Center Gas'!Q26</f>
-        <v>34216.315999999999</v>
-      </c>
-      <c r="R4" s="82">
-        <f>'Data Center Gas'!R26</f>
-        <v>34238.228000000003</v>
-      </c>
-      <c r="S4" s="82">
-        <f>'Data Center Gas'!S26</f>
-        <v>34258.498999999996</v>
-      </c>
-      <c r="T4" s="82">
-        <f>'Data Center Gas'!T26</f>
-        <v>34281.084999999999</v>
-      </c>
-      <c r="U4" s="82">
-        <f>'Data Center Gas'!U26</f>
-        <v>34301.161999999997</v>
-      </c>
-      <c r="V4" s="82">
-        <f>'Data Center Gas'!V26</f>
-        <v>34321.178</v>
-      </c>
-      <c r="W4" s="82">
-        <f>'Data Center Gas'!W26</f>
-        <v>34340.084000000003</v>
-      </c>
-      <c r="X4" s="82">
-        <f>'Data Center Gas'!X26</f>
-        <v>34359.432999999997</v>
-      </c>
-      <c r="Y4" s="82">
-        <f>'Data Center Gas'!Y26</f>
-        <v>34379.940999999999</v>
-      </c>
-      <c r="Z4" s="82">
-        <f>'Data Center Gas'!Z26</f>
-        <v>34400.097000000002</v>
-      </c>
-      <c r="AA4" s="82">
-        <f>'Data Center Gas'!AA26</f>
-        <v>34419.017999999996</v>
-      </c>
-      <c r="AB4" s="82">
-        <f>'Data Center Gas'!AB26</f>
-        <v>34439.06</v>
+      <c r="C4" s="64">
+        <f>'Data Center Gas'!D27</f>
+        <v>18508.008000000002</v>
+      </c>
+      <c r="D4" s="64">
+        <f>'Data Center Gas'!E27</f>
+        <v>22540.969000000001</v>
+      </c>
+      <c r="E4" s="64">
+        <f>'Data Center Gas'!F27</f>
+        <v>26559.125</v>
+      </c>
+      <c r="F4" s="64">
+        <f>'Data Center Gas'!G27</f>
+        <v>30576.868999999999</v>
+      </c>
+      <c r="G4" s="64">
+        <f>'Data Center Gas'!H27</f>
+        <v>40595.394999999997</v>
+      </c>
+      <c r="H4" s="64">
+        <f>'Data Center Gas'!I27</f>
+        <v>50615.290999999997</v>
+      </c>
+      <c r="I4" s="64">
+        <f>'Data Center Gas'!J27</f>
+        <v>50634.760999999999</v>
+      </c>
+      <c r="J4" s="64">
+        <f>'Data Center Gas'!K27</f>
+        <v>50655.343999999997</v>
+      </c>
+      <c r="K4" s="64">
+        <f>'Data Center Gas'!L27</f>
+        <v>50676.552000000003</v>
+      </c>
+      <c r="L4" s="64">
+        <f>'Data Center Gas'!M27</f>
+        <v>50700.095000000001</v>
+      </c>
+      <c r="M4" s="64">
+        <f>'Data Center Gas'!N27</f>
+        <v>50722.014000000003</v>
+      </c>
+      <c r="N4" s="64">
+        <f>'Data Center Gas'!O27</f>
+        <v>50744.811999999998</v>
+      </c>
+      <c r="O4" s="64">
+        <f>'Data Center Gas'!P27</f>
+        <v>50769.997000000003</v>
+      </c>
+      <c r="P4" s="64">
+        <f>'Data Center Gas'!Q27</f>
+        <v>50793.459000000003</v>
+      </c>
+      <c r="Q4" s="64">
+        <f>'Data Center Gas'!R27</f>
+        <v>50816.315999999999</v>
+      </c>
+      <c r="R4" s="64">
+        <f>'Data Center Gas'!S27</f>
+        <v>50838.228000000003</v>
+      </c>
+      <c r="S4" s="64">
+        <f>'Data Center Gas'!T27</f>
+        <v>50858.498999999996</v>
+      </c>
+      <c r="T4" s="64">
+        <f>'Data Center Gas'!U27</f>
+        <v>50881.084999999999</v>
+      </c>
+      <c r="U4" s="64">
+        <f>'Data Center Gas'!V27</f>
+        <v>50901.161999999997</v>
+      </c>
+      <c r="V4" s="64">
+        <f>'Data Center Gas'!W27</f>
+        <v>50921.178</v>
+      </c>
+      <c r="W4" s="64">
+        <f>'Data Center Gas'!X27</f>
+        <v>50940.084000000003</v>
+      </c>
+      <c r="X4" s="64">
+        <f>'Data Center Gas'!Y27</f>
+        <v>50959.432999999997</v>
+      </c>
+      <c r="Y4" s="64">
+        <f>'Data Center Gas'!Z27</f>
+        <v>50979.940999999999</v>
+      </c>
+      <c r="Z4" s="64">
+        <f>'Data Center Gas'!AA27</f>
+        <v>51000.097000000002</v>
+      </c>
+      <c r="AA4" s="64">
+        <f>'Data Center Gas'!AB27</f>
+        <v>51019.017999999996</v>
+      </c>
+      <c r="AB4" s="64">
+        <f>'Data Center Gas'!AC27</f>
+        <v>51039.06</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.25">
@@ -31595,105 +31859,105 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="73" t="s">
         <v>959</v>
       </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
+      <c r="I1" s="73"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
+      <c r="M1" s="73"/>
+      <c r="N1" s="73"/>
+      <c r="O1" s="73"/>
+      <c r="P1" s="73"/>
+      <c r="Q1" s="73"/>
+      <c r="R1" s="73"/>
+      <c r="S1" s="73"/>
+      <c r="T1" s="73"/>
+      <c r="U1" s="73"/>
     </row>
     <row r="2" spans="1:21" ht="39" x14ac:dyDescent="0.25">
       <c r="A2" s="63" t="s">
         <v>958</v>
       </c>
-      <c r="B2" s="64" t="s">
+      <c r="B2" s="74" t="s">
         <v>957</v>
       </c>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
-      <c r="I2" s="68"/>
-      <c r="J2" s="68"/>
-      <c r="K2" s="68"/>
-      <c r="L2" s="68"/>
-      <c r="M2" s="68"/>
-      <c r="N2" s="68"/>
-      <c r="O2" s="65"/>
-      <c r="P2" s="64" t="s">
+      <c r="C2" s="75"/>
+      <c r="D2" s="75"/>
+      <c r="E2" s="75"/>
+      <c r="F2" s="75"/>
+      <c r="G2" s="75"/>
+      <c r="H2" s="75"/>
+      <c r="I2" s="75"/>
+      <c r="J2" s="75"/>
+      <c r="K2" s="75"/>
+      <c r="L2" s="75"/>
+      <c r="M2" s="75"/>
+      <c r="N2" s="75"/>
+      <c r="O2" s="76"/>
+      <c r="P2" s="74" t="s">
         <v>956</v>
       </c>
-      <c r="Q2" s="65"/>
-      <c r="R2" s="64" t="s">
+      <c r="Q2" s="76"/>
+      <c r="R2" s="74" t="s">
         <v>955</v>
       </c>
-      <c r="S2" s="68"/>
-      <c r="T2" s="68"/>
-      <c r="U2" s="65"/>
+      <c r="S2" s="75"/>
+      <c r="T2" s="75"/>
+      <c r="U2" s="76"/>
     </row>
     <row r="3" spans="1:21" ht="39" x14ac:dyDescent="0.25">
       <c r="A3" s="63" t="s">
         <v>954</v>
       </c>
-      <c r="B3" s="64" t="s">
+      <c r="B3" s="74" t="s">
         <v>86</v>
       </c>
-      <c r="C3" s="65"/>
-      <c r="D3" s="64" t="s">
+      <c r="C3" s="76"/>
+      <c r="D3" s="74" t="s">
         <v>953</v>
       </c>
-      <c r="E3" s="65"/>
-      <c r="F3" s="64" t="s">
+      <c r="E3" s="76"/>
+      <c r="F3" s="74" t="s">
         <v>44</v>
       </c>
-      <c r="G3" s="65"/>
-      <c r="H3" s="64" t="s">
+      <c r="G3" s="76"/>
+      <c r="H3" s="74" t="s">
         <v>952</v>
       </c>
-      <c r="I3" s="65"/>
-      <c r="J3" s="64" t="s">
+      <c r="I3" s="76"/>
+      <c r="J3" s="74" t="s">
         <v>951</v>
       </c>
-      <c r="K3" s="65"/>
-      <c r="L3" s="64" t="s">
+      <c r="K3" s="76"/>
+      <c r="L3" s="74" t="s">
         <v>950</v>
       </c>
-      <c r="M3" s="65"/>
-      <c r="N3" s="64" t="s">
+      <c r="M3" s="76"/>
+      <c r="N3" s="74" t="s">
         <v>949</v>
       </c>
-      <c r="O3" s="65"/>
-      <c r="P3" s="64" t="s">
+      <c r="O3" s="76"/>
+      <c r="P3" s="74" t="s">
         <v>948</v>
       </c>
-      <c r="Q3" s="65"/>
-      <c r="R3" s="64" t="s">
+      <c r="Q3" s="76"/>
+      <c r="R3" s="74" t="s">
         <v>947</v>
       </c>
-      <c r="S3" s="65"/>
-      <c r="T3" s="64" t="s">
+      <c r="S3" s="76"/>
+      <c r="T3" s="74" t="s">
         <v>946</v>
       </c>
-      <c r="U3" s="65"/>
+      <c r="U3" s="76"/>
     </row>
     <row r="4" spans="1:21" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A4" s="63" t="s">
@@ -35791,32 +36055,33 @@
       </c>
     </row>
     <row r="67" spans="1:21" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="66" t="s">
+      <c r="A67" s="72" t="s">
         <v>887</v>
       </c>
-      <c r="B67" s="66"/>
-      <c r="C67" s="66"/>
-      <c r="D67" s="66"/>
-      <c r="E67" s="66"/>
-      <c r="F67" s="66"/>
-      <c r="G67" s="66"/>
-      <c r="H67" s="66"/>
-      <c r="I67" s="66"/>
-      <c r="J67" s="66"/>
-      <c r="K67" s="66"/>
-      <c r="L67" s="66"/>
-      <c r="M67" s="66"/>
-      <c r="N67" s="66"/>
-      <c r="O67" s="66"/>
-      <c r="P67" s="66"/>
-      <c r="Q67" s="66"/>
-      <c r="R67" s="66"/>
-      <c r="S67" s="66"/>
-      <c r="T67" s="66"/>
-      <c r="U67" s="66"/>
+      <c r="B67" s="72"/>
+      <c r="C67" s="72"/>
+      <c r="D67" s="72"/>
+      <c r="E67" s="72"/>
+      <c r="F67" s="72"/>
+      <c r="G67" s="72"/>
+      <c r="H67" s="72"/>
+      <c r="I67" s="72"/>
+      <c r="J67" s="72"/>
+      <c r="K67" s="72"/>
+      <c r="L67" s="72"/>
+      <c r="M67" s="72"/>
+      <c r="N67" s="72"/>
+      <c r="O67" s="72"/>
+      <c r="P67" s="72"/>
+      <c r="Q67" s="72"/>
+      <c r="R67" s="72"/>
+      <c r="S67" s="72"/>
+      <c r="T67" s="72"/>
+      <c r="U67" s="72"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A67:U67"/>
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="B2:O2"/>
     <mergeCell ref="P2:Q2"/>
@@ -35831,7 +36096,6 @@
     <mergeCell ref="P3:Q3"/>
     <mergeCell ref="R3:S3"/>
     <mergeCell ref="T3:U3"/>
-    <mergeCell ref="A67:U67"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup scale="37" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -48528,43 +48792,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="86" t="s">
         <v>369</v>
       </c>
-      <c r="B1" s="75"/>
+      <c r="B1" s="83"/>
     </row>
     <row r="2" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="74" t="s">
+      <c r="A2" s="82" t="s">
         <v>370</v>
       </c>
-      <c r="B2" s="75"/>
-      <c r="C2" s="75"/>
-      <c r="D2" s="75"/>
-      <c r="E2" s="75"/>
-      <c r="F2" s="75"/>
-      <c r="G2" s="75"/>
+      <c r="B2" s="83"/>
+      <c r="C2" s="83"/>
+      <c r="D2" s="83"/>
+      <c r="E2" s="83"/>
+      <c r="F2" s="83"/>
+      <c r="G2" s="83"/>
     </row>
     <row r="3" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="17"/>
-      <c r="B3" s="69" t="s">
+      <c r="B3" s="77" t="s">
         <v>371</v>
       </c>
-      <c r="C3" s="70"/>
-      <c r="D3" s="70"/>
-      <c r="E3" s="70"/>
-      <c r="F3" s="70"/>
-      <c r="G3" s="70"/>
+      <c r="C3" s="78"/>
+      <c r="D3" s="78"/>
+      <c r="E3" s="78"/>
+      <c r="F3" s="78"/>
+      <c r="G3" s="78"/>
     </row>
     <row r="4" spans="1:7" ht="23.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A4" s="17"/>
       <c r="B4" s="19"/>
-      <c r="C4" s="71" t="s">
+      <c r="C4" s="79" t="s">
         <v>372</v>
       </c>
-      <c r="D4" s="72"/>
-      <c r="E4" s="72"/>
-      <c r="F4" s="72"/>
-      <c r="G4" s="73"/>
+      <c r="D4" s="80"/>
+      <c r="E4" s="80"/>
+      <c r="F4" s="80"/>
+      <c r="G4" s="81"/>
     </row>
     <row r="5" spans="1:7" ht="46.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="20"/>
@@ -53085,15 +53349,15 @@
       <c r="G220" s="25"/>
     </row>
     <row r="221" spans="1:7" s="6" customFormat="1" ht="206.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A221" s="76" t="s">
+      <c r="A221" s="84" t="s">
         <v>523</v>
       </c>
-      <c r="B221" s="77"/>
-      <c r="C221" s="77"/>
-      <c r="D221" s="77"/>
-      <c r="E221" s="77"/>
-      <c r="F221" s="77"/>
-      <c r="G221" s="77"/>
+      <c r="B221" s="85"/>
+      <c r="C221" s="85"/>
+      <c r="D221" s="85"/>
+      <c r="E221" s="85"/>
+      <c r="F221" s="85"/>
+      <c r="G221" s="85"/>
     </row>
     <row r="222" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>

</xml_diff>